<commit_message>
Update of curtailed energy calcualtion. Scenario preparation
</commit_message>
<xml_diff>
--- a/data/Fertig - 1.a_MS_misch_base/1.a_MS_misch_grid-reduced/Power_BusInfo.xlsx
+++ b/data/Fertig - 1.a_MS_misch_base/1.a_MS_misch_grid-reduced/Power_BusInfo.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="R:\01_Modelle\2025-02-24_DyLeR-20\Scenarios_1.a\1.a_MS_misch\1.a_MS_misch_base\1.a_MS_misch_grid-reduced\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GIT\LEGO-Pyomo\data\Fertig - 1.a_MS_misch_base\1.a_MS_misch_grid-reduced\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{686F95D6-0397-43EB-8CF7-66D1CC13E3F4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C7CE1ACC-2837-4B3B-BEA2-A018883CB72F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="36230" yWindow="2730" windowWidth="28800" windowHeight="15240" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ScenarioA" sheetId="1" r:id="rId1"/>
@@ -1369,18 +1369,21 @@
     <tabColor rgb="FF008080"/>
   </sheetPr>
   <dimension ref="A1:S192"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.703125" defaultRowHeight="14.35" x14ac:dyDescent="0.5"/>
   <cols>
-    <col min="1" max="1" width="5.54296875" customWidth="1"/>
-    <col min="2" max="2" width="19.7265625" customWidth="1"/>
-    <col min="3" max="12" width="15.7265625" customWidth="1"/>
-    <col min="13" max="14" width="20.1796875" customWidth="1"/>
-    <col min="15" max="16" width="15.7265625" customWidth="1"/>
-    <col min="17" max="17" width="18.7265625" customWidth="1"/>
-    <col min="18" max="19" width="24.54296875" customWidth="1"/>
+    <col min="1" max="1" width="5.52734375" customWidth="1"/>
+    <col min="2" max="2" width="19.703125" customWidth="1"/>
+    <col min="3" max="6" width="15.703125" customWidth="1"/>
+    <col min="7" max="7" width="16.46875" bestFit="1" customWidth="1"/>
+    <col min="8" max="9" width="21.5859375" bestFit="1" customWidth="1"/>
+    <col min="10" max="12" width="15.703125" customWidth="1"/>
+    <col min="13" max="14" width="20.17578125" customWidth="1"/>
+    <col min="15" max="16" width="15.703125" customWidth="1"/>
+    <col min="17" max="17" width="18.703125" customWidth="1"/>
+    <col min="18" max="19" width="24.52734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:19" ht="24" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="1" spans="1:19" ht="24" customHeight="1" x14ac:dyDescent="0.85">
       <c r="A1" s="1"/>
       <c r="B1" s="2" t="s">
         <v>0</v>
@@ -1403,7 +1406,7 @@
       <c r="R1" s="1"/>
       <c r="S1" s="1"/>
     </row>
-    <row r="2" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:19" x14ac:dyDescent="0.5">
       <c r="B2" s="3" t="s">
         <v>1</v>
       </c>
@@ -1411,7 +1414,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:19" x14ac:dyDescent="0.5">
       <c r="A3" s="5" t="s">
         <v>3</v>
       </c>
@@ -1470,7 +1473,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="4" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:19" x14ac:dyDescent="0.5">
       <c r="A4" s="6" t="s">
         <v>20</v>
       </c>
@@ -1529,7 +1532,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="5" spans="1:19" ht="45" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:19" ht="45" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A5" s="7"/>
       <c r="B5" s="7" t="s">
         <v>37</v>
@@ -1586,7 +1589,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="6" spans="1:19" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:19" ht="30" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A6" s="8"/>
       <c r="B6" s="8" t="s">
         <v>51</v>
@@ -1639,7 +1642,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="7" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:19" x14ac:dyDescent="0.5">
       <c r="A7" s="9"/>
       <c r="B7" s="9" t="s">
         <v>54</v>
@@ -1692,7 +1695,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="8" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:19" x14ac:dyDescent="0.5">
       <c r="A8" s="10"/>
       <c r="B8" s="11"/>
       <c r="C8" s="12" t="s">
@@ -1739,7 +1742,7 @@
       <c r="R8" s="17"/>
       <c r="S8" s="17"/>
     </row>
-    <row r="9" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:19" x14ac:dyDescent="0.5">
       <c r="A9" s="10"/>
       <c r="B9" s="11"/>
       <c r="C9" s="12" t="s">
@@ -1790,7 +1793,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="10" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:19" x14ac:dyDescent="0.5">
       <c r="A10" s="10"/>
       <c r="B10" s="11"/>
       <c r="C10" s="12" t="s">
@@ -1841,7 +1844,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="11" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:19" x14ac:dyDescent="0.5">
       <c r="A11" s="10"/>
       <c r="B11" s="11"/>
       <c r="C11" s="12" t="s">
@@ -1892,7 +1895,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="12" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:19" x14ac:dyDescent="0.5">
       <c r="A12" s="10"/>
       <c r="B12" s="11"/>
       <c r="C12" s="12" t="s">
@@ -1943,7 +1946,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="13" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:19" x14ac:dyDescent="0.5">
       <c r="A13" s="10"/>
       <c r="B13" s="11"/>
       <c r="C13" s="12" t="s">
@@ -1994,7 +1997,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="14" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:19" x14ac:dyDescent="0.5">
       <c r="A14" s="10"/>
       <c r="B14" s="11"/>
       <c r="C14" s="12" t="s">
@@ -2045,7 +2048,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="15" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:19" x14ac:dyDescent="0.5">
       <c r="A15" s="10"/>
       <c r="B15" s="11"/>
       <c r="C15" s="12" t="s">
@@ -2096,7 +2099,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="16" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:19" x14ac:dyDescent="0.5">
       <c r="A16" s="10"/>
       <c r="B16" s="11"/>
       <c r="C16" s="12" t="s">
@@ -2147,7 +2150,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="17" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:19" x14ac:dyDescent="0.5">
       <c r="A17" s="10"/>
       <c r="B17" s="11"/>
       <c r="C17" s="12" t="s">
@@ -2198,7 +2201,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="18" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:19" x14ac:dyDescent="0.5">
       <c r="A18" s="10"/>
       <c r="B18" s="11"/>
       <c r="C18" s="12" t="s">
@@ -2249,7 +2252,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="19" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:19" x14ac:dyDescent="0.5">
       <c r="A19" s="10"/>
       <c r="B19" s="11"/>
       <c r="C19" s="12" t="s">
@@ -2300,7 +2303,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="20" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:19" x14ac:dyDescent="0.5">
       <c r="A20" s="10"/>
       <c r="B20" s="11"/>
       <c r="C20" s="12" t="s">
@@ -2351,7 +2354,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="21" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:19" x14ac:dyDescent="0.5">
       <c r="A21" s="10"/>
       <c r="B21" s="11"/>
       <c r="C21" s="12" t="s">
@@ -2402,7 +2405,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="22" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:19" x14ac:dyDescent="0.5">
       <c r="A22" s="10"/>
       <c r="B22" s="11"/>
       <c r="C22" s="12" t="s">
@@ -2453,7 +2456,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="23" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:19" x14ac:dyDescent="0.5">
       <c r="A23" s="10"/>
       <c r="B23" s="11"/>
       <c r="C23" s="12" t="s">
@@ -2504,7 +2507,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="24" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:19" x14ac:dyDescent="0.5">
       <c r="A24" s="10"/>
       <c r="B24" s="11"/>
       <c r="C24" s="12" t="s">
@@ -2555,7 +2558,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="25" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:19" x14ac:dyDescent="0.5">
       <c r="A25" s="10"/>
       <c r="B25" s="11"/>
       <c r="C25" s="12" t="s">
@@ -2606,7 +2609,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="26" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:19" x14ac:dyDescent="0.5">
       <c r="A26" s="10"/>
       <c r="B26" s="11"/>
       <c r="C26" s="12" t="s">
@@ -2657,7 +2660,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="27" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:19" x14ac:dyDescent="0.5">
       <c r="A27" s="10"/>
       <c r="B27" s="11"/>
       <c r="C27" s="12" t="s">
@@ -2708,7 +2711,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="28" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:19" x14ac:dyDescent="0.5">
       <c r="A28" s="10"/>
       <c r="B28" s="11"/>
       <c r="C28" s="12" t="s">
@@ -2759,7 +2762,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="29" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:19" x14ac:dyDescent="0.5">
       <c r="A29" s="10"/>
       <c r="B29" s="11"/>
       <c r="C29" s="12" t="s">
@@ -2810,7 +2813,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="30" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:19" x14ac:dyDescent="0.5">
       <c r="A30" s="10"/>
       <c r="B30" s="11"/>
       <c r="C30" s="12" t="s">
@@ -2861,7 +2864,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="31" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:19" x14ac:dyDescent="0.5">
       <c r="A31" s="10"/>
       <c r="B31" s="11"/>
       <c r="C31" s="12" t="s">
@@ -2912,7 +2915,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="32" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:19" x14ac:dyDescent="0.5">
       <c r="A32" s="10"/>
       <c r="B32" s="11"/>
       <c r="C32" s="12" t="s">
@@ -2963,7 +2966,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="33" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:19" x14ac:dyDescent="0.5">
       <c r="A33" s="10"/>
       <c r="B33" s="11"/>
       <c r="C33" s="12" t="s">
@@ -3014,7 +3017,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="34" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:19" x14ac:dyDescent="0.5">
       <c r="A34" s="10"/>
       <c r="B34" s="11"/>
       <c r="C34" s="12" t="s">
@@ -3065,7 +3068,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="35" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:19" x14ac:dyDescent="0.5">
       <c r="A35" s="10"/>
       <c r="B35" s="11"/>
       <c r="C35" s="12" t="s">
@@ -3116,7 +3119,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="36" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:19" x14ac:dyDescent="0.5">
       <c r="A36" s="10"/>
       <c r="B36" s="11"/>
       <c r="C36" s="12" t="s">
@@ -3167,7 +3170,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="37" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:19" x14ac:dyDescent="0.5">
       <c r="A37" s="10"/>
       <c r="B37" s="11"/>
       <c r="C37" s="12" t="s">
@@ -3218,7 +3221,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="38" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:19" x14ac:dyDescent="0.5">
       <c r="A38" s="10"/>
       <c r="B38" s="11"/>
       <c r="C38" s="12" t="s">
@@ -3269,7 +3272,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="39" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:19" x14ac:dyDescent="0.5">
       <c r="A39" s="10"/>
       <c r="B39" s="11"/>
       <c r="C39" s="12" t="s">
@@ -3320,7 +3323,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="40" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:19" x14ac:dyDescent="0.5">
       <c r="A40" s="10"/>
       <c r="B40" s="11"/>
       <c r="C40" s="12" t="s">
@@ -3371,7 +3374,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="41" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:19" x14ac:dyDescent="0.5">
       <c r="A41" s="10"/>
       <c r="B41" s="11"/>
       <c r="C41" s="12" t="s">
@@ -3422,7 +3425,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="42" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:19" x14ac:dyDescent="0.5">
       <c r="A42" s="10"/>
       <c r="B42" s="11"/>
       <c r="C42" s="12" t="s">
@@ -3473,7 +3476,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="43" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:19" x14ac:dyDescent="0.5">
       <c r="A43" s="10"/>
       <c r="B43" s="11"/>
       <c r="C43" s="12" t="s">
@@ -3524,7 +3527,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="44" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:19" x14ac:dyDescent="0.5">
       <c r="A44" s="10"/>
       <c r="B44" s="11"/>
       <c r="C44" s="12" t="s">
@@ -3575,7 +3578,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="45" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:19" x14ac:dyDescent="0.5">
       <c r="A45" s="10"/>
       <c r="B45" s="11"/>
       <c r="C45" s="12" t="s">
@@ -3626,7 +3629,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="46" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:19" x14ac:dyDescent="0.5">
       <c r="A46" s="10"/>
       <c r="B46" s="11"/>
       <c r="C46" s="12" t="s">
@@ -3677,7 +3680,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="47" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:19" x14ac:dyDescent="0.5">
       <c r="A47" s="10"/>
       <c r="B47" s="11"/>
       <c r="C47" s="12" t="s">
@@ -3728,7 +3731,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="48" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:19" x14ac:dyDescent="0.5">
       <c r="A48" s="10"/>
       <c r="B48" s="11"/>
       <c r="C48" s="12" t="s">
@@ -3779,7 +3782,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="49" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:19" x14ac:dyDescent="0.5">
       <c r="A49" s="10"/>
       <c r="B49" s="11"/>
       <c r="C49" s="12" t="s">
@@ -3830,7 +3833,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="50" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:19" x14ac:dyDescent="0.5">
       <c r="A50" s="10"/>
       <c r="B50" s="11"/>
       <c r="C50" s="12" t="s">
@@ -3881,7 +3884,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="51" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:19" x14ac:dyDescent="0.5">
       <c r="A51" s="10"/>
       <c r="B51" s="11"/>
       <c r="C51" s="12" t="s">
@@ -3932,7 +3935,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="52" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:19" x14ac:dyDescent="0.5">
       <c r="A52" s="10"/>
       <c r="B52" s="11"/>
       <c r="C52" s="12" t="s">
@@ -3983,7 +3986,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="53" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:19" x14ac:dyDescent="0.5">
       <c r="A53" s="10"/>
       <c r="B53" s="11"/>
       <c r="C53" s="12" t="s">
@@ -4034,7 +4037,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="54" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:19" x14ac:dyDescent="0.5">
       <c r="A54" s="10"/>
       <c r="B54" s="11"/>
       <c r="C54" s="12" t="s">
@@ -4085,7 +4088,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="55" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:19" x14ac:dyDescent="0.5">
       <c r="A55" s="10"/>
       <c r="B55" s="11"/>
       <c r="C55" s="12" t="s">
@@ -4136,7 +4139,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="56" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:19" x14ac:dyDescent="0.5">
       <c r="A56" s="10"/>
       <c r="B56" s="11"/>
       <c r="C56" s="12" t="s">
@@ -4187,7 +4190,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="57" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:19" x14ac:dyDescent="0.5">
       <c r="A57" s="10"/>
       <c r="B57" s="11"/>
       <c r="C57" s="12" t="s">
@@ -4238,7 +4241,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="58" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:19" x14ac:dyDescent="0.5">
       <c r="A58" s="10"/>
       <c r="B58" s="11"/>
       <c r="C58" s="12" t="s">
@@ -4289,7 +4292,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="59" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:19" x14ac:dyDescent="0.5">
       <c r="A59" s="10"/>
       <c r="B59" s="11"/>
       <c r="C59" s="12" t="s">
@@ -4340,7 +4343,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="60" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:19" x14ac:dyDescent="0.5">
       <c r="A60" s="10"/>
       <c r="B60" s="11"/>
       <c r="C60" s="12" t="s">
@@ -4391,7 +4394,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="61" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:19" x14ac:dyDescent="0.5">
       <c r="A61" s="10"/>
       <c r="B61" s="11"/>
       <c r="C61" s="12" t="s">
@@ -4442,7 +4445,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="62" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:19" x14ac:dyDescent="0.5">
       <c r="A62" s="10"/>
       <c r="B62" s="11"/>
       <c r="C62" s="12" t="s">
@@ -4493,7 +4496,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="63" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:19" x14ac:dyDescent="0.5">
       <c r="A63" s="10"/>
       <c r="B63" s="11"/>
       <c r="C63" s="12" t="s">
@@ -4544,7 +4547,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="64" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:19" x14ac:dyDescent="0.5">
       <c r="A64" s="10"/>
       <c r="B64" s="11"/>
       <c r="C64" s="12" t="s">
@@ -4595,7 +4598,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="65" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:19" x14ac:dyDescent="0.5">
       <c r="A65" s="10"/>
       <c r="B65" s="11"/>
       <c r="C65" s="12" t="s">
@@ -4646,7 +4649,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="66" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:19" x14ac:dyDescent="0.5">
       <c r="A66" s="10"/>
       <c r="B66" s="11"/>
       <c r="C66" s="12" t="s">
@@ -4697,7 +4700,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="67" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:19" x14ac:dyDescent="0.5">
       <c r="A67" s="10"/>
       <c r="B67" s="11"/>
       <c r="C67" s="12" t="s">
@@ -4748,7 +4751,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="68" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:19" x14ac:dyDescent="0.5">
       <c r="A68" s="10"/>
       <c r="B68" s="11"/>
       <c r="C68" s="12" t="s">
@@ -4799,7 +4802,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="69" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:19" x14ac:dyDescent="0.5">
       <c r="A69" s="10"/>
       <c r="B69" s="11"/>
       <c r="C69" s="12" t="s">
@@ -4850,7 +4853,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="70" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:19" x14ac:dyDescent="0.5">
       <c r="A70" s="10"/>
       <c r="B70" s="11"/>
       <c r="C70" s="12" t="s">
@@ -4901,7 +4904,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="71" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:19" x14ac:dyDescent="0.5">
       <c r="A71" s="10"/>
       <c r="B71" s="11"/>
       <c r="C71" s="12" t="s">
@@ -4952,7 +4955,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="72" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:19" x14ac:dyDescent="0.5">
       <c r="A72" s="10"/>
       <c r="B72" s="11"/>
       <c r="C72" s="12" t="s">
@@ -5003,7 +5006,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="73" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:19" x14ac:dyDescent="0.5">
       <c r="A73" s="10"/>
       <c r="B73" s="11"/>
       <c r="C73" s="12" t="s">
@@ -5054,7 +5057,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="74" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:19" x14ac:dyDescent="0.5">
       <c r="A74" s="10"/>
       <c r="B74" s="11"/>
       <c r="C74" s="12" t="s">
@@ -5105,7 +5108,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="75" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:19" x14ac:dyDescent="0.5">
       <c r="A75" s="10"/>
       <c r="B75" s="11"/>
       <c r="C75" s="12" t="s">
@@ -5156,7 +5159,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="76" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:19" x14ac:dyDescent="0.5">
       <c r="A76" s="10"/>
       <c r="B76" s="11"/>
       <c r="C76" s="12" t="s">
@@ -5207,7 +5210,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="77" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:19" x14ac:dyDescent="0.5">
       <c r="A77" s="10"/>
       <c r="B77" s="11"/>
       <c r="C77" s="12" t="s">
@@ -5258,7 +5261,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="78" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:19" x14ac:dyDescent="0.5">
       <c r="A78" s="10"/>
       <c r="B78" s="11"/>
       <c r="C78" s="12" t="s">
@@ -5309,7 +5312,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="79" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:19" x14ac:dyDescent="0.5">
       <c r="A79" s="10"/>
       <c r="B79" s="11"/>
       <c r="C79" s="12" t="s">
@@ -5360,7 +5363,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="80" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:19" x14ac:dyDescent="0.5">
       <c r="A80" s="10"/>
       <c r="B80" s="11"/>
       <c r="C80" s="12" t="s">
@@ -5411,7 +5414,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="81" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:19" x14ac:dyDescent="0.5">
       <c r="A81" s="10"/>
       <c r="B81" s="11"/>
       <c r="C81" s="12" t="s">
@@ -5462,7 +5465,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="82" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:19" x14ac:dyDescent="0.5">
       <c r="A82" s="10"/>
       <c r="B82" s="11"/>
       <c r="C82" s="12" t="s">
@@ -5513,7 +5516,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="83" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:19" x14ac:dyDescent="0.5">
       <c r="A83" s="10"/>
       <c r="B83" s="11"/>
       <c r="C83" s="12" t="s">
@@ -5564,7 +5567,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="84" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:19" x14ac:dyDescent="0.5">
       <c r="A84" s="10"/>
       <c r="B84" s="11"/>
       <c r="C84" s="12" t="s">
@@ -5615,7 +5618,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="85" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:19" x14ac:dyDescent="0.5">
       <c r="A85" s="10"/>
       <c r="B85" s="11"/>
       <c r="C85" s="12" t="s">
@@ -5666,7 +5669,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="86" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:19" x14ac:dyDescent="0.5">
       <c r="A86" s="10"/>
       <c r="B86" s="11"/>
       <c r="C86" s="12" t="s">
@@ -5717,7 +5720,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="87" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:19" x14ac:dyDescent="0.5">
       <c r="A87" s="10"/>
       <c r="B87" s="11"/>
       <c r="C87" s="12" t="s">
@@ -5768,7 +5771,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="88" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:19" x14ac:dyDescent="0.5">
       <c r="A88" s="10"/>
       <c r="B88" s="11"/>
       <c r="C88" s="12" t="s">
@@ -5819,7 +5822,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="89" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:19" x14ac:dyDescent="0.5">
       <c r="A89" s="10"/>
       <c r="B89" s="11"/>
       <c r="C89" s="12" t="s">
@@ -5870,7 +5873,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="90" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:19" x14ac:dyDescent="0.5">
       <c r="A90" s="10"/>
       <c r="B90" s="11"/>
       <c r="C90" s="12" t="s">
@@ -5921,7 +5924,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="91" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:19" x14ac:dyDescent="0.5">
       <c r="A91" s="10"/>
       <c r="B91" s="11"/>
       <c r="C91" s="12" t="s">
@@ -5972,7 +5975,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="92" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:19" x14ac:dyDescent="0.5">
       <c r="A92" s="10"/>
       <c r="B92" s="11"/>
       <c r="C92" s="12" t="s">
@@ -6023,7 +6026,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="93" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:19" x14ac:dyDescent="0.5">
       <c r="A93" s="10"/>
       <c r="B93" s="11"/>
       <c r="C93" s="12" t="s">
@@ -6074,7 +6077,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="94" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:19" x14ac:dyDescent="0.5">
       <c r="A94" s="10"/>
       <c r="B94" s="11"/>
       <c r="C94" s="12" t="s">
@@ -6125,7 +6128,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="95" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:19" x14ac:dyDescent="0.5">
       <c r="A95" s="10"/>
       <c r="B95" s="11"/>
       <c r="C95" s="12" t="s">
@@ -6176,7 +6179,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="96" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:19" x14ac:dyDescent="0.5">
       <c r="A96" s="10"/>
       <c r="B96" s="11"/>
       <c r="C96" s="12" t="s">
@@ -6227,7 +6230,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="97" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:19" x14ac:dyDescent="0.5">
       <c r="A97" s="10"/>
       <c r="B97" s="11"/>
       <c r="C97" s="12" t="s">
@@ -6278,7 +6281,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="98" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:19" x14ac:dyDescent="0.5">
       <c r="A98" s="10"/>
       <c r="B98" s="11"/>
       <c r="C98" s="12" t="s">
@@ -6329,7 +6332,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="99" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:19" x14ac:dyDescent="0.5">
       <c r="A99" s="10"/>
       <c r="B99" s="11"/>
       <c r="C99" s="12" t="s">
@@ -6380,7 +6383,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="100" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:19" x14ac:dyDescent="0.5">
       <c r="A100" s="10"/>
       <c r="B100" s="11"/>
       <c r="C100" s="12" t="s">
@@ -6431,7 +6434,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="101" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:19" x14ac:dyDescent="0.5">
       <c r="A101" s="10"/>
       <c r="B101" s="11"/>
       <c r="C101" s="12" t="s">
@@ -6482,7 +6485,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="102" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="102" spans="1:19" x14ac:dyDescent="0.5">
       <c r="A102" s="10"/>
       <c r="B102" s="11"/>
       <c r="C102" s="12" t="s">
@@ -6533,7 +6536,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="103" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:19" x14ac:dyDescent="0.5">
       <c r="A103" s="10"/>
       <c r="B103" s="11"/>
       <c r="C103" s="12" t="s">
@@ -6584,7 +6587,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="104" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="104" spans="1:19" x14ac:dyDescent="0.5">
       <c r="A104" s="10"/>
       <c r="B104" s="11"/>
       <c r="C104" s="12" t="s">
@@ -6635,7 +6638,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="105" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="105" spans="1:19" x14ac:dyDescent="0.5">
       <c r="A105" s="10"/>
       <c r="B105" s="11"/>
       <c r="C105" s="12" t="s">
@@ -6686,7 +6689,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="106" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="106" spans="1:19" x14ac:dyDescent="0.5">
       <c r="A106" s="10"/>
       <c r="B106" s="11"/>
       <c r="C106" s="12" t="s">
@@ -6737,7 +6740,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="107" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="107" spans="1:19" x14ac:dyDescent="0.5">
       <c r="A107" s="10"/>
       <c r="B107" s="11"/>
       <c r="C107" s="12" t="s">
@@ -6788,7 +6791,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="108" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="108" spans="1:19" x14ac:dyDescent="0.5">
       <c r="A108" s="10"/>
       <c r="B108" s="11"/>
       <c r="C108" s="12" t="s">
@@ -6839,7 +6842,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="109" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="109" spans="1:19" x14ac:dyDescent="0.5">
       <c r="A109" s="10"/>
       <c r="B109" s="11"/>
       <c r="C109" s="12" t="s">
@@ -6890,7 +6893,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="110" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="110" spans="1:19" x14ac:dyDescent="0.5">
       <c r="A110" s="10"/>
       <c r="B110" s="11"/>
       <c r="C110" s="12" t="s">
@@ -6941,7 +6944,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="111" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="111" spans="1:19" x14ac:dyDescent="0.5">
       <c r="A111" s="10"/>
       <c r="B111" s="11"/>
       <c r="C111" s="12" t="s">
@@ -6992,7 +6995,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="112" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="112" spans="1:19" x14ac:dyDescent="0.5">
       <c r="A112" s="10"/>
       <c r="B112" s="11"/>
       <c r="C112" s="12" t="s">
@@ -7043,7 +7046,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="113" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="113" spans="1:19" x14ac:dyDescent="0.5">
       <c r="A113" s="10"/>
       <c r="B113" s="11"/>
       <c r="C113" s="12" t="s">
@@ -7094,7 +7097,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="114" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="114" spans="1:19" x14ac:dyDescent="0.5">
       <c r="A114" s="10"/>
       <c r="B114" s="11"/>
       <c r="C114" s="12" t="s">
@@ -7145,7 +7148,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="115" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="115" spans="1:19" x14ac:dyDescent="0.5">
       <c r="A115" s="10"/>
       <c r="B115" s="11"/>
       <c r="C115" s="12" t="s">
@@ -7196,7 +7199,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="116" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="116" spans="1:19" x14ac:dyDescent="0.5">
       <c r="A116" s="10"/>
       <c r="B116" s="11"/>
       <c r="C116" s="12" t="s">
@@ -7247,7 +7250,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="117" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="117" spans="1:19" x14ac:dyDescent="0.5">
       <c r="A117" s="10"/>
       <c r="B117" s="11"/>
       <c r="C117" s="12" t="s">
@@ -7298,7 +7301,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="118" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="118" spans="1:19" x14ac:dyDescent="0.5">
       <c r="A118" s="10"/>
       <c r="B118" s="11"/>
       <c r="C118" s="12" t="s">
@@ -7349,7 +7352,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="119" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="119" spans="1:19" x14ac:dyDescent="0.5">
       <c r="A119" s="10"/>
       <c r="B119" s="11"/>
       <c r="C119" s="12" t="s">
@@ -7400,7 +7403,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="120" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="120" spans="1:19" x14ac:dyDescent="0.5">
       <c r="A120" s="10"/>
       <c r="B120" s="11"/>
       <c r="C120" s="12" t="s">
@@ -7451,7 +7454,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="121" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="121" spans="1:19" x14ac:dyDescent="0.5">
       <c r="A121" s="10"/>
       <c r="B121" s="11"/>
       <c r="C121" s="12" t="s">
@@ -7502,7 +7505,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="122" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="122" spans="1:19" x14ac:dyDescent="0.5">
       <c r="A122" s="10"/>
       <c r="B122" s="11"/>
       <c r="C122" s="12" t="s">
@@ -7553,7 +7556,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="123" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="123" spans="1:19" x14ac:dyDescent="0.5">
       <c r="A123" s="10"/>
       <c r="B123" s="11"/>
       <c r="C123" s="12" t="s">
@@ -7604,7 +7607,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="124" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="124" spans="1:19" x14ac:dyDescent="0.5">
       <c r="A124" s="10"/>
       <c r="B124" s="11"/>
       <c r="C124" s="12" t="s">
@@ -7655,7 +7658,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="125" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="125" spans="1:19" x14ac:dyDescent="0.5">
       <c r="A125" s="10"/>
       <c r="B125" s="11"/>
       <c r="C125" s="12" t="s">
@@ -7706,7 +7709,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="126" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="126" spans="1:19" x14ac:dyDescent="0.5">
       <c r="A126" s="10"/>
       <c r="B126" s="11"/>
       <c r="C126" s="12" t="s">
@@ -7757,7 +7760,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="127" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="127" spans="1:19" x14ac:dyDescent="0.5">
       <c r="A127" s="10"/>
       <c r="B127" s="11"/>
       <c r="C127" s="12" t="s">
@@ -7808,7 +7811,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="128" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="128" spans="1:19" x14ac:dyDescent="0.5">
       <c r="A128" s="10"/>
       <c r="B128" s="11"/>
       <c r="C128" s="12" t="s">
@@ -7859,7 +7862,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="129" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="129" spans="1:19" x14ac:dyDescent="0.5">
       <c r="A129" s="10"/>
       <c r="B129" s="11"/>
       <c r="C129" s="12" t="s">
@@ -7910,7 +7913,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="130" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="130" spans="1:19" x14ac:dyDescent="0.5">
       <c r="A130" s="10"/>
       <c r="B130" s="11"/>
       <c r="C130" s="12" t="s">
@@ -7961,7 +7964,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="131" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="131" spans="1:19" x14ac:dyDescent="0.5">
       <c r="A131" s="10"/>
       <c r="B131" s="11"/>
       <c r="C131" s="12" t="s">
@@ -8012,7 +8015,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="132" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="132" spans="1:19" x14ac:dyDescent="0.5">
       <c r="A132" s="10"/>
       <c r="B132" s="11"/>
       <c r="C132" s="12" t="s">
@@ -8063,7 +8066,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="133" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="133" spans="1:19" x14ac:dyDescent="0.5">
       <c r="A133" s="10"/>
       <c r="B133" s="11"/>
       <c r="C133" s="12" t="s">
@@ -8114,7 +8117,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="134" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="134" spans="1:19" x14ac:dyDescent="0.5">
       <c r="A134" s="10"/>
       <c r="B134" s="11"/>
       <c r="C134" s="12" t="s">
@@ -8165,7 +8168,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="135" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="135" spans="1:19" x14ac:dyDescent="0.5">
       <c r="A135" s="10"/>
       <c r="B135" s="11"/>
       <c r="C135" s="12" t="s">
@@ -8216,7 +8219,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="136" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="136" spans="1:19" x14ac:dyDescent="0.5">
       <c r="A136" s="10"/>
       <c r="B136" s="11"/>
       <c r="C136" s="12" t="s">
@@ -8267,7 +8270,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="137" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="137" spans="1:19" x14ac:dyDescent="0.5">
       <c r="A137" s="10"/>
       <c r="B137" s="11"/>
       <c r="C137" s="12" t="s">
@@ -8318,7 +8321,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="138" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="138" spans="1:19" x14ac:dyDescent="0.5">
       <c r="A138" s="10"/>
       <c r="B138" s="11"/>
       <c r="C138" s="12" t="s">
@@ -8369,7 +8372,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="139" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="139" spans="1:19" x14ac:dyDescent="0.5">
       <c r="A139" s="10"/>
       <c r="B139" s="11"/>
       <c r="C139" s="12" t="s">
@@ -8420,7 +8423,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="140" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="140" spans="1:19" x14ac:dyDescent="0.5">
       <c r="A140" s="10"/>
       <c r="B140" s="11"/>
       <c r="C140" s="12" t="s">
@@ -8471,7 +8474,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="141" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="141" spans="1:19" x14ac:dyDescent="0.5">
       <c r="A141" s="10"/>
       <c r="B141" s="11"/>
       <c r="C141" s="12" t="s">
@@ -8522,7 +8525,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="142" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="142" spans="1:19" x14ac:dyDescent="0.5">
       <c r="A142" s="10"/>
       <c r="B142" s="11"/>
       <c r="C142" s="12" t="s">
@@ -8573,7 +8576,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="143" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="143" spans="1:19" x14ac:dyDescent="0.5">
       <c r="A143" s="10"/>
       <c r="B143" s="11"/>
       <c r="C143" s="12" t="s">
@@ -8624,7 +8627,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="144" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="144" spans="1:19" x14ac:dyDescent="0.5">
       <c r="A144" s="10"/>
       <c r="B144" s="11"/>
       <c r="C144" s="12" t="s">
@@ -8675,7 +8678,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="145" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="145" spans="1:19" x14ac:dyDescent="0.5">
       <c r="A145" s="10"/>
       <c r="B145" s="11"/>
       <c r="C145" s="12" t="s">
@@ -8726,7 +8729,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="146" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="146" spans="1:19" x14ac:dyDescent="0.5">
       <c r="A146" s="10"/>
       <c r="B146" s="11"/>
       <c r="C146" s="12" t="s">
@@ -8777,7 +8780,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="147" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="147" spans="1:19" x14ac:dyDescent="0.5">
       <c r="A147" s="10"/>
       <c r="B147" s="11"/>
       <c r="C147" s="12" t="s">
@@ -8828,7 +8831,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="148" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="148" spans="1:19" x14ac:dyDescent="0.5">
       <c r="A148" s="10"/>
       <c r="B148" s="11"/>
       <c r="C148" s="12" t="s">
@@ -8879,7 +8882,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="149" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="149" spans="1:19" x14ac:dyDescent="0.5">
       <c r="A149" s="10"/>
       <c r="B149" s="11"/>
       <c r="C149" s="12" t="s">
@@ -8930,7 +8933,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="150" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="150" spans="1:19" x14ac:dyDescent="0.5">
       <c r="A150" s="10"/>
       <c r="B150" s="11"/>
       <c r="C150" s="12" t="s">
@@ -8981,7 +8984,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="151" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="151" spans="1:19" x14ac:dyDescent="0.5">
       <c r="A151" s="10"/>
       <c r="B151" s="11"/>
       <c r="C151" s="12" t="s">
@@ -9032,7 +9035,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="152" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="152" spans="1:19" x14ac:dyDescent="0.5">
       <c r="A152" s="10"/>
       <c r="B152" s="11"/>
       <c r="C152" s="12" t="s">
@@ -9083,7 +9086,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="153" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="153" spans="1:19" x14ac:dyDescent="0.5">
       <c r="A153" s="10"/>
       <c r="B153" s="11"/>
       <c r="C153" s="12" t="s">
@@ -9134,7 +9137,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="154" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="154" spans="1:19" x14ac:dyDescent="0.5">
       <c r="A154" s="10"/>
       <c r="B154" s="11"/>
       <c r="C154" s="12" t="s">
@@ -9185,7 +9188,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="155" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="155" spans="1:19" x14ac:dyDescent="0.5">
       <c r="A155" s="10"/>
       <c r="B155" s="11"/>
       <c r="C155" s="12" t="s">
@@ -9236,7 +9239,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="156" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="156" spans="1:19" x14ac:dyDescent="0.5">
       <c r="A156" s="10"/>
       <c r="B156" s="11"/>
       <c r="C156" s="12" t="s">
@@ -9287,7 +9290,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="157" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="157" spans="1:19" x14ac:dyDescent="0.5">
       <c r="A157" s="10"/>
       <c r="B157" s="11"/>
       <c r="C157" s="12" t="s">
@@ -9338,7 +9341,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="158" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="158" spans="1:19" x14ac:dyDescent="0.5">
       <c r="A158" s="10"/>
       <c r="B158" s="11"/>
       <c r="C158" s="12" t="s">
@@ -9389,7 +9392,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="159" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="159" spans="1:19" x14ac:dyDescent="0.5">
       <c r="A159" s="10"/>
       <c r="B159" s="11"/>
       <c r="C159" s="12" t="s">
@@ -9440,7 +9443,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="160" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="160" spans="1:19" x14ac:dyDescent="0.5">
       <c r="A160" s="10"/>
       <c r="B160" s="11"/>
       <c r="C160" s="12" t="s">
@@ -9491,7 +9494,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="161" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="161" spans="1:19" x14ac:dyDescent="0.5">
       <c r="A161" s="10"/>
       <c r="B161" s="11"/>
       <c r="C161" s="12" t="s">
@@ -9542,7 +9545,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="162" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="162" spans="1:19" x14ac:dyDescent="0.5">
       <c r="A162" s="10"/>
       <c r="B162" s="11"/>
       <c r="C162" s="12" t="s">
@@ -9593,7 +9596,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="163" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="163" spans="1:19" x14ac:dyDescent="0.5">
       <c r="A163" s="10"/>
       <c r="B163" s="11"/>
       <c r="C163" s="12" t="s">
@@ -9644,7 +9647,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="164" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="164" spans="1:19" x14ac:dyDescent="0.5">
       <c r="A164" s="10"/>
       <c r="B164" s="11"/>
       <c r="C164" s="12" t="s">
@@ -9695,7 +9698,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="165" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="165" spans="1:19" x14ac:dyDescent="0.5">
       <c r="A165" s="10"/>
       <c r="B165" s="11"/>
       <c r="C165" s="12" t="s">
@@ -9746,7 +9749,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="166" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="166" spans="1:19" x14ac:dyDescent="0.5">
       <c r="A166" s="10"/>
       <c r="B166" s="11"/>
       <c r="C166" s="12" t="s">
@@ -9797,7 +9800,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="167" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="167" spans="1:19" x14ac:dyDescent="0.5">
       <c r="A167" s="10"/>
       <c r="B167" s="11"/>
       <c r="C167" s="12" t="s">
@@ -9848,7 +9851,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="168" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="168" spans="1:19" x14ac:dyDescent="0.5">
       <c r="A168" s="10"/>
       <c r="B168" s="11"/>
       <c r="C168" s="12" t="s">
@@ -9899,7 +9902,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="169" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="169" spans="1:19" x14ac:dyDescent="0.5">
       <c r="A169" s="10"/>
       <c r="B169" s="11"/>
       <c r="C169" s="12" t="s">
@@ -9950,7 +9953,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="170" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="170" spans="1:19" x14ac:dyDescent="0.5">
       <c r="A170" s="10"/>
       <c r="B170" s="11"/>
       <c r="C170" s="12" t="s">
@@ -10001,7 +10004,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="171" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="171" spans="1:19" x14ac:dyDescent="0.5">
       <c r="A171" s="10"/>
       <c r="B171" s="11"/>
       <c r="C171" s="12" t="s">
@@ -10052,7 +10055,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="172" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="172" spans="1:19" x14ac:dyDescent="0.5">
       <c r="A172" s="10"/>
       <c r="B172" s="11"/>
       <c r="C172" s="12" t="s">
@@ -10103,7 +10106,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="173" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="173" spans="1:19" x14ac:dyDescent="0.5">
       <c r="A173" s="10"/>
       <c r="B173" s="11"/>
       <c r="C173" s="12" t="s">
@@ -10154,7 +10157,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="174" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="174" spans="1:19" x14ac:dyDescent="0.5">
       <c r="A174" s="10"/>
       <c r="B174" s="11"/>
       <c r="C174" s="12" t="s">
@@ -10205,7 +10208,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="175" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="175" spans="1:19" x14ac:dyDescent="0.5">
       <c r="A175" s="10"/>
       <c r="B175" s="11"/>
       <c r="C175" s="12" t="s">
@@ -10256,7 +10259,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="176" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="176" spans="1:19" x14ac:dyDescent="0.5">
       <c r="A176" s="10"/>
       <c r="B176" s="11"/>
       <c r="C176" s="12" t="s">
@@ -10307,7 +10310,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="177" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="177" spans="1:19" x14ac:dyDescent="0.5">
       <c r="A177" s="10"/>
       <c r="B177" s="11"/>
       <c r="C177" s="12" t="s">
@@ -10358,7 +10361,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="178" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="178" spans="1:19" x14ac:dyDescent="0.5">
       <c r="A178" s="10"/>
       <c r="B178" s="11"/>
       <c r="C178" s="12" t="s">
@@ -10409,7 +10412,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="179" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="179" spans="1:19" x14ac:dyDescent="0.5">
       <c r="A179" s="10"/>
       <c r="B179" s="11"/>
       <c r="C179" s="12" t="s">
@@ -10460,7 +10463,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="180" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="180" spans="1:19" x14ac:dyDescent="0.5">
       <c r="A180" s="10"/>
       <c r="B180" s="11"/>
       <c r="C180" s="12" t="s">
@@ -10511,7 +10514,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="181" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="181" spans="1:19" x14ac:dyDescent="0.5">
       <c r="A181" s="10"/>
       <c r="B181" s="11"/>
       <c r="C181" s="12" t="s">
@@ -10562,7 +10565,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="182" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="182" spans="1:19" x14ac:dyDescent="0.5">
       <c r="A182" s="10"/>
       <c r="B182" s="11"/>
       <c r="C182" s="12" t="s">
@@ -10613,7 +10616,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="183" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="183" spans="1:19" x14ac:dyDescent="0.5">
       <c r="A183" s="10"/>
       <c r="B183" s="11"/>
       <c r="C183" s="12" t="s">
@@ -10664,7 +10667,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="184" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="184" spans="1:19" x14ac:dyDescent="0.5">
       <c r="A184" s="10"/>
       <c r="B184" s="11"/>
       <c r="C184" s="12" t="s">
@@ -10715,7 +10718,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="185" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="185" spans="1:19" x14ac:dyDescent="0.5">
       <c r="A185" s="10"/>
       <c r="B185" s="11"/>
       <c r="C185" s="12" t="s">
@@ -10766,7 +10769,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="186" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="186" spans="1:19" x14ac:dyDescent="0.5">
       <c r="A186" s="10"/>
       <c r="B186" s="11"/>
       <c r="C186" s="12" t="s">
@@ -10817,7 +10820,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="187" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="187" spans="1:19" x14ac:dyDescent="0.5">
       <c r="A187" s="10"/>
       <c r="B187" s="11"/>
       <c r="C187" s="12" t="s">
@@ -10868,7 +10871,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="188" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="188" spans="1:19" x14ac:dyDescent="0.5">
       <c r="A188" s="10"/>
       <c r="B188" s="11"/>
       <c r="C188" s="12" t="s">
@@ -10919,7 +10922,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="189" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="189" spans="1:19" x14ac:dyDescent="0.5">
       <c r="A189" s="10"/>
       <c r="B189" s="11"/>
       <c r="C189" s="12" t="s">
@@ -10970,7 +10973,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="190" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="190" spans="1:19" x14ac:dyDescent="0.5">
       <c r="A190" s="10"/>
       <c r="B190" s="11"/>
       <c r="C190" s="12" t="s">
@@ -11021,7 +11024,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="191" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="191" spans="1:19" x14ac:dyDescent="0.5">
       <c r="A191" s="10"/>
       <c r="B191" s="11"/>
       <c r="C191" s="12" t="s">
@@ -11072,7 +11075,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="192" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="192" spans="1:19" x14ac:dyDescent="0.5">
       <c r="A192" s="10"/>
       <c r="B192" s="11"/>
       <c r="C192" s="12" t="s">

</xml_diff>